<commit_message>
Add the glossary term Specimen
Glossaire v1, B31: Active again, so Specimen is published in the clinical
glossary (FR definition only; no EN or NL yet). Reverts the previous
commit.
</commit_message>
<xml_diff>
--- a/input/Glossaire CareSets V1.xlsx
+++ b/input/Glossaire CareSets V1.xlsx
@@ -7511,10 +7511,8 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0" t="inlineStr">
-        <is>
-          <t>Inactive</t>
-        </is>
+      <c r="B31" s="0" t="s">
+        <v>1</v>
       </c>
       <c r="C31" s="0" t="s">
         <v>193</v>

</xml_diff>